<commit_message>
Model revamp to include production shocks successful
</commit_message>
<xml_diff>
--- a/data/initial_state_2026.xlsx
+++ b/data/initial_state_2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="14540"/>
+    <workbookView windowWidth="30240" windowHeight="14540" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="global.pars" sheetId="1" r:id="rId1"/>
@@ -12534,166 +12534,166 @@
         <v>236</v>
       </c>
       <c r="F30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="G30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="H30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="I30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="J30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="K30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="L30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="M30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="N30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="O30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="P30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Q30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="R30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="S30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="T30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="U30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="V30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="W30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="X30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Y30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Z30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AA30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AB30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AC30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AD30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AE30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AF30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AG30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AH30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AI30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AJ30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AK30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AL30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AM30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AN30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AO30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AP30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AQ30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AR30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AS30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AT30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AU30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AV30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AW30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AX30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AY30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AZ30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BA30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BB30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BC30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BD30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BE30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BF30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BG30">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31" spans="1:59">
@@ -12710,166 +12710,166 @@
         <v>236</v>
       </c>
       <c r="F31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="G31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="H31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="I31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="J31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="K31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="L31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="M31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="N31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="O31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="P31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Q31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="R31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="S31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="T31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="U31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="V31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="W31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="X31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Y31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Z31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AA31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AB31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AC31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AD31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AE31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AF31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AG31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AH31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AI31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AJ31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AK31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AL31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AM31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AN31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AO31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AP31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AQ31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AR31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AS31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AT31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AU31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AV31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AW31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AX31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AY31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="AZ31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BA31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BB31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BC31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BD31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BE31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BF31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="BG31">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32" spans="1:59">

</xml_diff>